<commit_message>
feat: complete Bid for C branding + redesigned registration
- Added BrandHeader component (4 variants: live, scoreboard, admin, team)
- Branding on all screens: LiveAuctionScreen, ScoreboardScreen, AdminScreen, TeamScreen
- Logo glow effect + fade-in animation on live screen
- Tagline: Bid Smart. Code Fast. Win Big.
- Redesigned Team Registration with split layout
  - Left: branding + event description + rules
  - Right: registration form
  - Navy background, gold accents, white text
  - Footer with About, How it Works, Winning Criteria
- Added Sound Settings collapsible panel with per-sound toggles
- Added file upload for sound files
- Updated README with comprehensive documentation
</commit_message>
<xml_diff>
--- a/auction-quiz/docs/quiz-questions.xlsx
+++ b/auction-quiz/docs/quiz-questions.xlsx
@@ -401,458 +401,436 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
-        <v>question_text</v>
+        <v>difficulty</v>
       </c>
       <c r="B1" t="str">
-        <v>options</v>
+        <v>file_path</v>
       </c>
       <c r="C1" t="str">
-        <v>difficulty</v>
+        <v>reward_points</v>
       </c>
       <c r="D1" t="str">
-        <v>reward_points</v>
+        <v>time_limit</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>What is the capital of France?</v>
+        <v>easy</v>
       </c>
       <c r="B2" t="str">
-        <v>["Paris","London","Berlin","Madrid"]</v>
-      </c>
-      <c r="C2" t="str">
-        <v>easy</v>
+        <v>easy/easy_01_switch_fallthrough.txt</v>
+      </c>
+      <c r="C2">
+        <v>10</v>
       </c>
       <c r="D2">
-        <v>10</v>
+        <v>60</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>What is 2 + 2 * 2?</v>
+        <v>easy</v>
       </c>
       <c r="B3" t="str">
-        <v>["6","8","4","10"]</v>
-      </c>
-      <c r="C3" t="str">
-        <v>easy</v>
+        <v>easy/easy_02_uninitialized_var.txt</v>
+      </c>
+      <c r="C3">
+        <v>10</v>
       </c>
       <c r="D3">
-        <v>10</v>
+        <v>60</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>Which is the largest planet in our solar system?</v>
+        <v>easy</v>
       </c>
       <c r="B4" t="str">
-        <v>["Jupiter","Saturn","Earth","Mars"]</v>
-      </c>
-      <c r="C4" t="str">
-        <v>easy</v>
+        <v>easy/easy_03_macro_square.txt</v>
+      </c>
+      <c r="C4">
+        <v>10</v>
       </c>
       <c r="D4">
-        <v>10</v>
+        <v>60</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>H2O is commonly known as what?</v>
+        <v>easy</v>
       </c>
       <c r="B5" t="str">
-        <v>["Water","Salt","Oxygen","Sugar"]</v>
-      </c>
-      <c r="C5" t="str">
-        <v>easy</v>
+        <v>easy/easy_04_printf_return.txt</v>
+      </c>
+      <c r="C5">
+        <v>10</v>
       </c>
       <c r="D5">
-        <v>10</v>
+        <v>60</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>How many days are there in a leap year?</v>
+        <v>easy</v>
       </c>
       <c r="B6" t="str">
-        <v>["366","365","364","367"]</v>
-      </c>
-      <c r="C6" t="str">
-        <v>easy</v>
+        <v>easy/easy_05_string_literal_segfault.txt</v>
+      </c>
+      <c r="C6">
+        <v>15</v>
       </c>
       <c r="D6">
-        <v>10</v>
+        <v>90</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>Name the process by which plants make their food.</v>
+        <v>easy</v>
       </c>
       <c r="B7" t="str">
-        <v/>
-      </c>
-      <c r="C7" t="str">
-        <v>easy</v>
+        <v>easy/easy_06_pointer_increment.txt</v>
+      </c>
+      <c r="C7">
+        <v>15</v>
       </c>
       <c r="D7">
-        <v>10</v>
+        <v>90</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>How many continents are there on Earth?</v>
+        <v>easy</v>
       </c>
       <c r="B8" t="str">
-        <v>["7","5","6","8"]</v>
-      </c>
-      <c r="C8" t="str">
-        <v>easy</v>
+        <v>easy/easy_07_scanf_missing_ampersand.txt</v>
+      </c>
+      <c r="C8">
+        <v>10</v>
       </c>
       <c r="D8">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>easy</v>
+      </c>
+      <c r="B9" t="str">
+        <v>easy/easy_08_static_local_var.txt</v>
+      </c>
+      <c r="C9">
         <v>10</v>
       </c>
-    </row>
-    <row r="9" xml:space="preserve">
-      <c r="A9" t="str" xml:space="preserve">
-        <v xml:space="preserve">What does this print?
-```
-print(2 + 3)
-```</v>
-      </c>
-      <c r="B9" t="str">
-        <v>["5","23","6","Error"]</v>
-      </c>
-      <c r="C9" t="str">
-        <v>easy</v>
-      </c>
       <c r="D9">
-        <v>10</v>
+        <v>60</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>Which device is used to point and click on a computer?</v>
+        <v>easy</v>
       </c>
       <c r="B10" t="str">
-        <v>["Mouse","Keyboard","Monitor","Printer"]</v>
-      </c>
-      <c r="C10" t="str">
-        <v>easy</v>
+        <v>easy/easy_09_semicolon_while.txt</v>
+      </c>
+      <c r="C10">
+        <v>10</v>
       </c>
       <c r="D10">
-        <v>10</v>
+        <v>60</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>What is the first element in the periodic table?</v>
+        <v>easy</v>
       </c>
       <c r="B11" t="str">
-        <v>["Hydrogen","Helium","Oxygen","Carbon"]</v>
-      </c>
-      <c r="C11" t="str">
-        <v>easy</v>
+        <v>easy/easy_10_array_off_by_one.txt</v>
+      </c>
+      <c r="C11">
+        <v>15</v>
       </c>
       <c r="D11">
-        <v>10</v>
+        <v>60</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>What is decimal 10 in binary?</v>
+        <v>medium</v>
       </c>
       <c r="B12" t="str">
-        <v>["1010","1001","1100","101"]</v>
-      </c>
-      <c r="C12" t="str">
-        <v>medium</v>
+        <v>medium/med_01_dangling_stack_pointer.txt</v>
+      </c>
+      <c r="C12">
+        <v>25</v>
       </c>
       <c r="D12">
-        <v>25</v>
+        <v>120</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>What is the time complexity of binary search?</v>
+        <v>medium</v>
       </c>
       <c r="B13" t="str">
-        <v>["O(log n)","O(n)","O(n log n)","O(1)"]</v>
-      </c>
-      <c r="C13" t="str">
-        <v>medium</v>
+        <v>medium/med_02_sizeof_array_parameter.txt</v>
+      </c>
+      <c r="C13">
+        <v>25</v>
       </c>
       <c r="D13">
-        <v>25</v>
+        <v>120</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>Which data structure follows LIFO (last in, first out) order?</v>
+        <v>medium</v>
       </c>
       <c r="B14" t="str">
-        <v/>
-      </c>
-      <c r="C14" t="str">
-        <v>medium</v>
+        <v>medium/med_03_recursion_static.txt</v>
+      </c>
+      <c r="C14">
+        <v>25</v>
       </c>
       <c r="D14">
-        <v>25</v>
+        <v>120</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>Which SQL command fetches all rows from a table called teams?</v>
+        <v>medium</v>
       </c>
       <c r="B15" t="str">
-        <v>["SELECT * FROM teams","GET ALL teams","FETCH * teams","RETRIEVE teams"]</v>
-      </c>
-      <c r="C15" t="str">
-        <v>medium</v>
+        <v>medium/med_04_missing_null_terminator.txt</v>
+      </c>
+      <c r="C15">
+        <v>30</v>
       </c>
       <c r="D15">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="str">
+        <v>medium</v>
+      </c>
+      <c r="B16" t="str">
+        <v>medium/med_05_struct_padding.txt</v>
+      </c>
+      <c r="C16">
         <v>25</v>
       </c>
-    </row>
-    <row r="16" xml:space="preserve">
-      <c r="A16" t="str" xml:space="preserve">
-        <v xml:space="preserve">What is printed?
-```
-for i in range(3):
-    print(i)
-```</v>
-      </c>
-      <c r="B16" t="str">
-        <v>["0 1 2","1 2 3","0 1 2 3","Error"]</v>
-      </c>
-      <c r="C16" t="str">
-        <v>medium</v>
-      </c>
       <c r="D16">
-        <v>25</v>
+        <v>120</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>Which is the largest ocean on Earth?</v>
+        <v>medium</v>
       </c>
       <c r="B17" t="str">
-        <v>["Pacific","Atlantic","Indian","Arctic"]</v>
-      </c>
-      <c r="C17" t="str">
-        <v>medium</v>
+        <v>medium/med_06_2d_array_pointers.txt</v>
+      </c>
+      <c r="C17">
+        <v>25</v>
       </c>
       <c r="D17">
-        <v>25</v>
+        <v>120</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>What does HTTP stand for?</v>
+        <v>medium</v>
       </c>
       <c r="B18" t="str">
-        <v/>
-      </c>
-      <c r="C18" t="str">
-        <v>medium</v>
+        <v>medium/med_07_malloc_memory_leak.txt</v>
+      </c>
+      <c r="C18">
+        <v>30</v>
       </c>
       <c r="D18">
-        <v>25</v>
+        <v>150</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>What is 15% of 200?</v>
+        <v>medium</v>
       </c>
       <c r="B19" t="str">
-        <v>["30","25","35","20"]</v>
-      </c>
-      <c r="C19" t="str">
-        <v>medium</v>
+        <v>medium/med_08_const_pointers.txt</v>
+      </c>
+      <c r="C19">
+        <v>25</v>
       </c>
       <c r="D19">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="str">
+        <v>medium</v>
+      </c>
+      <c r="B20" t="str">
+        <v>medium/med_09_bitwise_manipulation.txt</v>
+      </c>
+      <c r="C20">
         <v>25</v>
       </c>
-    </row>
-    <row r="20" xml:space="preserve">
-      <c r="A20" t="str" xml:space="preserve">
-        <v xml:space="preserve">What is printed?
-```
-x = [1, 2, 3]
-print(len(x))
-```</v>
-      </c>
-      <c r="B20" t="str">
-        <v>["3","2","6","Error"]</v>
-      </c>
-      <c r="C20" t="str">
-        <v>medium</v>
-      </c>
       <c r="D20">
-        <v>25</v>
+        <v>120</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>Name any two differences between RAM and ROM.</v>
+        <v>medium</v>
       </c>
       <c r="B21" t="str">
-        <v/>
-      </c>
-      <c r="C21" t="str">
-        <v>medium</v>
+        <v>medium/med_10_printf_type_mismatch.txt</v>
+      </c>
+      <c r="C21">
+        <v>30</v>
       </c>
       <c r="D21">
-        <v>25</v>
+        <v>120</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>Explain in 2-3 sentences why quicksort averages O(n log n) time.</v>
+        <v>hard</v>
       </c>
       <c r="B22" t="str">
-        <v/>
-      </c>
-      <c r="C22" t="str">
-        <v>hard</v>
+        <v>hard/hard_01_double_free.txt</v>
+      </c>
+      <c r="C22">
+        <v>50</v>
       </c>
       <c r="D22">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="str">
+        <v>hard</v>
+      </c>
+      <c r="B23" t="str">
+        <v>hard/hard_02_unsigned_loop_underflow.txt</v>
+      </c>
+      <c r="C23">
         <v>50</v>
       </c>
-    </row>
-    <row r="23" xml:space="preserve">
-      <c r="A23" t="str" xml:space="preserve">
-        <v xml:space="preserve">What is printed?
-```
-a = [1, 2, 3]
-b = a
-b.append(4)
-print(len(a))
-```</v>
-      </c>
-      <c r="B23" t="str">
-        <v>["4","3","Error","None"]</v>
-      </c>
-      <c r="C23" t="str">
-        <v>hard</v>
-      </c>
       <c r="D23">
-        <v>50</v>
+        <v>240</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>State the CAP theorem in one sentence.</v>
+        <v>hard</v>
       </c>
       <c r="B24" t="str">
-        <v/>
-      </c>
-      <c r="C24" t="str">
-        <v>hard</v>
+        <v>hard/hard_03_buffer_overflow_gets.txt</v>
+      </c>
+      <c r="C24">
+        <v>50</v>
       </c>
       <c r="D24">
-        <v>50</v>
+        <v>240</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>Which of these sorting algorithms is both stable and in-place?</v>
+        <v>hard</v>
       </c>
       <c r="B25" t="str">
-        <v>["Insertion sort","Merge sort","Quicksort","Heap sort"]</v>
-      </c>
-      <c r="C25" t="str">
-        <v>hard</v>
+        <v>hard/hard_04_complex_pointer_puzzle.txt</v>
+      </c>
+      <c r="C25">
+        <v>60</v>
       </c>
       <c r="D25">
-        <v>50</v>
+        <v>300</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>A train travels 120 km in 2 hours. A second train leaves 30 minutes later, same direction, at 80 km/h. After how many minutes does it catch up? Show your working.</v>
+        <v>hard</v>
       </c>
       <c r="B26" t="str">
-        <v/>
-      </c>
-      <c r="C26" t="str">
-        <v>hard</v>
+        <v>hard/hard_05_macro_double_increment.txt</v>
+      </c>
+      <c r="C26">
+        <v>50</v>
       </c>
       <c r="D26">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="str">
+        <v>hard</v>
+      </c>
+      <c r="B27" t="str">
+        <v>hard/hard_06_function_pointer_dispatch.txt</v>
+      </c>
+      <c r="C27">
         <v>50</v>
       </c>
-    </row>
-    <row r="27" xml:space="preserve">
-      <c r="A27" t="str" xml:space="preserve">
-        <v xml:space="preserve">What is printed?
-```
-def f(n):
-    return 1 if n &lt;= 1 else n * f(n - 1)
-print(f(4))
-```</v>
-      </c>
-      <c r="B27" t="str">
-        <v>["24","12","6","120"]</v>
-      </c>
-      <c r="C27" t="str">
-        <v>hard</v>
-      </c>
       <c r="D27">
-        <v>50</v>
+        <v>240</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>In binary, what is 1011 + 1101?</v>
+        <v>hard</v>
       </c>
       <c r="B28" t="str">
-        <v>["11000","10100","11100","10000"]</v>
-      </c>
-      <c r="C28" t="str">
-        <v>hard</v>
+        <v>hard/hard_07_realloc_pointer_leak.txt</v>
+      </c>
+      <c r="C28">
+        <v>50</v>
       </c>
       <c r="D28">
-        <v>50</v>
+        <v>240</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>Explain the difference between SQL INNER JOIN and LEFT JOIN with a small example.</v>
+        <v>hard</v>
       </c>
       <c r="B29" t="str">
-        <v/>
-      </c>
-      <c r="C29" t="str">
-        <v>hard</v>
+        <v>hard/hard_08_union_endianness.txt</v>
+      </c>
+      <c r="C29">
+        <v>50</v>
       </c>
       <c r="D29">
-        <v>50</v>
+        <v>240</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>In words: how would you rate-limit an API to 100 requests per minute per user? Mention where state lives.</v>
+        <v>hard</v>
       </c>
       <c r="B30" t="str">
-        <v/>
-      </c>
-      <c r="C30" t="str">
-        <v>hard</v>
+        <v>hard/hard_09_volatile_sig_atomic.txt</v>
+      </c>
+      <c r="C30">
+        <v>60</v>
       </c>
       <c r="D30">
-        <v>50</v>
+        <v>300</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>Name the treaty that ended World War I and the year it was signed.</v>
+        <v>hard</v>
       </c>
       <c r="B31" t="str">
-        <v/>
-      </c>
-      <c r="C31" t="str">
-        <v>hard</v>
+        <v>hard/hard_10_string_reverse_bug.txt</v>
+      </c>
+      <c r="C31">
+        <v>60</v>
       </c>
       <c r="D31">
-        <v>50</v>
+        <v>300</v>
       </c>
     </row>
   </sheetData>

</xml_diff>